<commit_message>
Use fully standardized Cohen's d in Tables 2 and 3.
</commit_message>
<xml_diff>
--- a/output/tables/Table3_Predictors_by_SNAP.xlsx
+++ b/output/tables/Table3_Predictors_by_SNAP.xlsx
@@ -72,7 +72,7 @@
     <t>0.18 (0.13, 0.23)</t>
   </si>
   <si>
-    <t>0.12</t>
+    <t>0.13</t>
   </si>
   <si>
     <t>&lt;0.001</t>
@@ -81,7 +81,7 @@
     <t>0.26 (0.22, 0.29)</t>
   </si>
   <si>
-    <t>0.18</t>
+    <t>0.19</t>
   </si>
   <si>
     <t>Embarrassment when paying with SNAP</t>
@@ -90,7 +90,7 @@
     <t>-0.11 (-0.14, -0.08)</t>
   </si>
   <si>
-    <t>-0.07</t>
+    <t>-0.09</t>
   </si>
   <si>
     <t>0.01 (-0.03, 0.05)</t>
@@ -108,19 +108,19 @@
     <t>-0.45 (-0.52, -0.39)</t>
   </si>
   <si>
-    <t>-0.31</t>
+    <t>-0.36</t>
   </si>
   <si>
     <t>-0.12 (-0.22, -0.03)</t>
   </si>
   <si>
-    <t>-0.08</t>
+    <t>-0.10</t>
   </si>
   <si>
     <t>0.01</t>
   </si>
   <si>
-    <t>Note. Coefficients are simple slopes (change in support per 1-unit increase in the predictor) from an OLS model with continuous predictors, SNAP participation, predictor×SNAP interactions, and covariates (age, gender, ethnicity, education, income, census region, children in household, state restriction status). Cohen's d = b / SD(support), the change in support in outcome SD units per 1-unit increase in the predictor. Standard errors clustered by state. Outcome: support for removing soft drinks and candy from SNAP-eligible purchases (1 = Strongly oppose to 5 = Strongly support). Unweighted. Complete-case analysis.</t>
+    <t>Note. Coefficients are simple slopes (change in support per 1-unit increase in the predictor) from an OLS model with continuous predictors, SNAP participation, predictor×SNAP interactions, and covariates (age, gender, ethnicity, education, income, census region, children in household, state restriction status). Cohen's d is the fully standardized effect: b × SD(predictor) / SD(support), using the analysis-sample SD of each predictor (common across SNAP groups) so effects are comparable across predictors and between Non-SNAP and SNAP. Standard errors clustered by state. Outcome: support for removing soft drinks and candy from SNAP-eligible purchases (1 = Strongly oppose to 5 = Strongly support). Unweighted. Complete-case analysis.</t>
   </si>
 </sst>
 </file>

</xml_diff>